<commit_message>
full refactoring of the vignette
</commit_message>
<xml_diff>
--- a/inst/templates/MalReBay_template_ampseq.xlsx
+++ b/inst/templates/MalReBay_template_ampseq.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Late Treatment Failures" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recurrent infections" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Additional" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -63,7 +63,19 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Alleles for marker cpmp: one column per allele (cpmp_allele_1, cpmp_allele_2, ...). Rename to your markers.</t>
+          <t xml:space="preserve">Alleles for marker/amplicon cpmp: one column per allele (cpmp_allele_1, cpmp_allele_2, ...). Rename to your corresponding markers.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D2" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Each allele is represented by its haplotype label (text), e.g. cpmp-1.</t>
         </r>
       </text>
     </comment>
@@ -121,7 +133,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Alleles for marker cpmp: one column per allele (cpmp_allele_1, cpmp_allele_2, ...). Rename to your markers.</t>
+          <t xml:space="preserve">Alleles for marker/amplicon cpmp: one column per allele (cpmp_allele_1, cpmp_allele_2, ...). Rename to your corresponding markers.</t>
         </r>
       </text>
     </comment>
@@ -130,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t xml:space="preserve">PatientID</t>
   </si>
@@ -237,22 +249,34 @@
     <t xml:space="preserve">ama1-D3-2</t>
   </si>
   <si>
+    <t xml:space="preserve">EXAMPLE-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpmp-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpp-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ama1-D3-7</t>
+  </si>
+  <si>
     <t xml:space="preserve">MalReBay data template: amplicon sequencing (AmpSeq)</t>
   </si>
   <si>
     <t xml:space="preserve">What to edit</t>
   </si>
   <si>
-    <t xml:space="preserve">1. On 'Late Treatment Failures', delete the grey example rows and enter one row per sample: a Day 0 row and a recurrence row for every patient with a recurrent infection.</t>
+    <t xml:space="preserve">1. On the 'Recurrent infections' sheet, replace the grey example rows with your data, one row per sample: a Day 0 row and a recurrence row for every patient with a recurrent infection.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. On 'Additional' (optional), delete the grey example row and enter Day 0 samples from other patients in the same study (e.g. patients without recurrence). They are used only to estimate background allele frequencies. Leave the sheet empty (headers only) if you have none.</t>
+    <t xml:space="preserve">2. On the 'Additional' sheet (optional), replace the grey example rows and enter Day 0 samples from other patients in the same study (e.g. patients without recurrence). They are used only to estimate background allele frequencies. Leave the sheet empty (headers only) if you have no data.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Rename / add / remove the marker columns to match your panel (see 'Allele columns' below). Both data sheets must have the same marker columns.</t>
+    <t xml:space="preserve">3. Rename / add / remove the marker columns to match your panel (see 'Allele columns' specifications below). Both data sheets must have the same marker columns.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Keep the sheet order: MalReBay reads the FIRST sheet as late failures and the SECOND as additional data, regardless of their names. Do not insert sheets before them.</t>
+    <t xml:space="preserve">4. Keep the sheet order: MalReBay reads the FIRST sheet as recurrent infections and the SECOND as additional data, regardless of their names. Do not insert sheets before them.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Run: import_data(filepath = "your_file.xlsx", marker_filepath = "your_marker_details.xlsx")</t>
@@ -297,7 +321,7 @@
     <t xml:space="preserve">• Name each allele column &lt;marker&gt;_allele_&lt;n&gt;, e.g. cpmp_allele_1, cpmp_allele_2, ... One column per allele observed in a sample; add as many as the highest number of alleles (multiplicity of infection) seen for that marker.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Marker names must match the marker_id column of the marker details file exactly (case-sensitive). Markers not found there are skipped with a message.</t>
+    <t xml:space="preserve">• Marker names must match the marker_id column of the marker details file exactly (case-sensitive). Markers not found there will be skipped with a message.</t>
   </si>
   <si>
     <t xml:space="preserve">• Fill alleles from the left (_1 first) and leave the remaining cells empty.</t>
@@ -315,31 +339,31 @@
     <t xml:space="preserve">• A separate xlsx with one row per marker and columns: marker_id, markertype, repeatlength, binning_method.</t>
   </si>
   <si>
-    <t xml:space="preserve">• MalReBay ships one with common markers: system.file("extdata", "makers_details.xlsx", package = "MalReBay"). Copy it and add rows for any markers of yours that are missing.</t>
+    <t xml:space="preserve">• MalReBay provides a file with common markers: system.file("extdata", "makers_details.xlsx", package = "MalReBay"). Copy it and add rows for any markers of yours that are missing.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend</t>
   </si>
   <si>
-    <t xml:space="preserve">Dark blue header</t>
+    <t xml:space="preserve">Dark header</t>
   </si>
   <si>
     <t xml:space="preserve">Required sample information columns</t>
   </si>
   <si>
-    <t xml:space="preserve">Light blue header</t>
+    <t xml:space="preserve">Light header</t>
   </si>
   <si>
     <t xml:space="preserve">Allele columns: rename/add/remove to match your panel</t>
   </si>
   <si>
-    <t xml:space="preserve">Grey italic rows</t>
+    <t xml:space="preserve">Grey rows</t>
   </si>
   <si>
     <t xml:space="preserve">Examples only: delete before running MalReBay</t>
   </si>
   <si>
-    <t xml:space="preserve">Hover over a column header on the data sheets for a short note.</t>
+    <t xml:space="preserve">Hover over the column headers on the data sheets for a short note.</t>
   </si>
 </sst>
 </file>
@@ -347,11 +371,51 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Aptos"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF432CA0"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF432CA0"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <b/>
     </font>
     <font>
       <sz val="10"/>
@@ -369,25 +433,6 @@
       <sz val="10"/>
       <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <b/>
     </font>
   </fonts>
   <fills count="4">
@@ -399,12 +444,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
+        <fgColor rgb="FF432CA0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
+        <fgColor rgb="FFD6CFF2"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -436,17 +481,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,21 +797,21 @@
     <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="13.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="13.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="12.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="14.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="14.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="14.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="11" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="11" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="12.715" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="12.715" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="12.715" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="12.715" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="12.715" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="12.715" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10864,21 +10920,21 @@
     <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="13.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="13.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="12.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="14.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="14.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="14.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.8575" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="11" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="11" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="12.715" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="12.715" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="12.715" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="12.715" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="12.715" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="12.715" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10970,24 +11026,38 @@
       <c r="R2" s="3"/>
     </row>
     <row r="3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
@@ -20953,53 +21023,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
@@ -21007,10 +21077,10 @@
         <v>0</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
@@ -21018,10 +21088,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
@@ -21029,7 +21099,7 @@
         <v>2</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>19</v>
@@ -21037,10 +21107,10 @@
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>20</v>
@@ -21048,81 +21118,81 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="s">
-        <v>63</v>
+      <c r="A29" s="10" t="s">
+        <v>67</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="s">
-        <v>65</v>
+      <c r="A30" s="11" t="s">
+        <v>69</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="s">
-        <v>67</v>
+      <c r="A31" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>